<commit_message>
Updated WebDriverUtility with overloaded waits and refactored POM pages for stability
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dell\Hybrid-FrameWork\ninza-crm-automation\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FD3FC71-AD42-46C0-9A49-1DC035BB770D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3408C53E-17D1-48AE-A2F0-AFB347484197}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="15">
   <si>
     <t>Campaign Name</t>
   </si>
@@ -68,6 +68,9 @@
   </si>
   <si>
     <t>Contact Name</t>
+  </si>
+  <si>
+    <t>Ashwin</t>
   </si>
 </sst>
 </file>
@@ -543,10 +546,10 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="B2">
-        <v>8130908100</v>
+        <v>8130908107</v>
       </c>
       <c r="C2" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
Added Lead module tests and improved existing CRM automation framework
- Added LeadsPage object repository
- Implemented CreateLeadTest, EditLeadTest, and DeleteLeadTest
- Added BrowserStackDemo test for campaign execution
- Enhanced BaseTest and WebDriverUtility for stability
- Updated CampaignsPage, ContactsPage, and HomePage locators/methods
- Improved contact tests (Create, Edit, Delete) for better reliability
- Updated TestData.xlsx and commonData.properties with new test data
- Added/updated testng.xml and reporting outputs
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dell\Hybrid-FrameWork\ninza-crm-automation\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3408C53E-17D1-48AE-A2F0-AFB347484197}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26F72667-0E0A-4EC1-8180-37A55AB32C4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -549,7 +549,7 @@
         <v>14</v>
       </c>
       <c r="B2">
-        <v>8130908107</v>
+        <v>9931061008</v>
       </c>
       <c r="C2" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
Refactor LeadsPage POM and add Excel utility
- Updated LeadsPage.java with professional low-level action methods and business flows
- Refactored createLead method to return Lead ID for better test reusability
- Added XlUtility.java for reading/writing test data from Excel
- Updated TestData.xlsx with new sample data
- Updated pom.xml and Maven metadata
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dell\Hybrid-FrameWork\ninza-crm-automation\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26F72667-0E0A-4EC1-8180-37A55AB32C4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB339D0C-3913-4795-B7C7-CBC4813D0F8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Campaigns" sheetId="1" r:id="rId1"/>
     <sheet name="Contacts" sheetId="2" r:id="rId2"/>
+    <sheet name="Leads" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="27">
   <si>
     <t>Campaign Name</t>
   </si>
@@ -71,13 +72,49 @@
   </si>
   <si>
     <t>Ashwin</t>
+  </si>
+  <si>
+    <t>Lead Name</t>
+  </si>
+  <si>
+    <t>Company</t>
+  </si>
+  <si>
+    <t>Lead Source</t>
+  </si>
+  <si>
+    <t>Lead Status</t>
+  </si>
+  <si>
+    <t>Industry</t>
+  </si>
+  <si>
+    <t>Phone</t>
+  </si>
+  <si>
+    <t>Rohit Verma</t>
+  </si>
+  <si>
+    <t>TechNova Solutions</t>
+  </si>
+  <si>
+    <t>Website</t>
+  </si>
+  <si>
+    <t>Contacted</t>
+  </si>
+  <si>
+    <t>IT Services</t>
+  </si>
+  <si>
+    <t>+91 9123456789</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -92,16 +129,29 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF333333"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -109,13 +159,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -578,4 +645,62 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82D6849F-7B86-4E10-8CE2-016D239A6825}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="11.81640625" customWidth="1"/>
+    <col min="2" max="2" width="17.6328125" customWidth="1"/>
+    <col min="3" max="3" width="15.1796875" customWidth="1"/>
+    <col min="4" max="4" width="11.36328125" customWidth="1"/>
+    <col min="5" max="5" width="15.1796875" customWidth="1"/>
+    <col min="6" max="6" width="14.90625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Refactor LeadsPage, tests, and add POJO & DataProvider
- Updated LeadsPage POM to accept Lead POJO and support createLead workflow
- Refactored CreateLeadTest and CreateCampaignTest for POJO-based data handling
- Added Lead POJO class in model package
- Added LeadsDataProvider class to provide Lead objects from Excel
- Updated TestData.xlsx with lead and campaign data
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dell\Hybrid-FrameWork\ninza-crm-automation\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB339D0C-3913-4795-B7C7-CBC4813D0F8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C9987B7-E69A-469B-9C53-FE537A60DE67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Campaigns" sheetId="1" r:id="rId1"/>
     <sheet name="Contacts" sheetId="2" r:id="rId2"/>
     <sheet name="Leads" sheetId="3" r:id="rId3"/>
+    <sheet name="CampaignData" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -27,10 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="27">
-  <si>
-    <t>Campaign Name</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="24">
   <si>
     <t>Target Size</t>
   </si>
@@ -47,9 +45,6 @@
     <t>this is great way to start a campaign</t>
   </si>
   <si>
-    <t>Ash</t>
-  </si>
-  <si>
     <t>dex</t>
   </si>
   <si>
@@ -74,9 +69,6 @@
     <t>Ashwin</t>
   </si>
   <si>
-    <t>Lead Name</t>
-  </si>
-  <si>
     <t>Company</t>
   </si>
   <si>
@@ -92,9 +84,6 @@
     <t>Phone</t>
   </si>
   <si>
-    <t>Rohit Verma</t>
-  </si>
-  <si>
     <t>TechNova Solutions</t>
   </si>
   <si>
@@ -108,6 +97,9 @@
   </si>
   <si>
     <t>+91 9123456789</t>
+  </si>
+  <si>
+    <t>CampaignName</t>
   </si>
 </sst>
 </file>
@@ -238,10 +230,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A9E8C391-7DCC-41C0-BBB9-5E3D8721855E}" name="Table1" displayName="Table1" ref="A1:D3" totalsRowShown="0" headerRowDxfId="1">
-  <autoFilter ref="A1:D3" xr:uid="{A9E8C391-7DCC-41C0-BBB9-5E3D8721855E}"/>
-  <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{80CCBB80-E6D3-43C6-9412-ABC098016D17}" name="Campaign Name"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A9E8C391-7DCC-41C0-BBB9-5E3D8721855E}" name="Table1" displayName="Table1" ref="A1:C3" totalsRowShown="0" headerRowDxfId="1">
+  <autoFilter ref="A1:C3" xr:uid="{A9E8C391-7DCC-41C0-BBB9-5E3D8721855E}"/>
+  <tableColumns count="3">
     <tableColumn id="2" xr3:uid="{180767D8-EC2D-4617-A851-893273784D2A}" name="Target Size"/>
     <tableColumn id="3" xr3:uid="{7EC7D0D4-C759-4AEE-BBE2-B7BAE18727BD}" name="Campaign Status"/>
     <tableColumn id="4" xr3:uid="{D674CE91-21D2-46C9-8A03-09743FA6976D}" name="Description"/>
@@ -526,16 +517,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
     <col min="2" max="2" width="9.90625" customWidth="1"/>
-    <col min="3" max="3" width="15.453125" customWidth="1"/>
+    <col min="3" max="3" width="32.90625" customWidth="1"/>
     <col min="4" max="4" width="30.36328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -545,36 +536,27 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>100</v>
+      </c>
+      <c r="B2" t="s">
         <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2">
-        <v>100</v>
       </c>
       <c r="C2" t="s">
         <v>4</v>
       </c>
-      <c r="D2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3">
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3">
         <v>50</v>
+      </c>
+      <c r="B3" t="s">
+        <v>3</v>
       </c>
       <c r="C3" t="s">
         <v>4</v>
-      </c>
-      <c r="D3" t="s">
-        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -599,44 +581,44 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B2">
         <v>9931061008</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B3">
         <v>9911021960</v>
       </c>
       <c r="C3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -649,55 +631,66 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82D6849F-7B86-4E10-8CE2-016D239A6825}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.81640625" customWidth="1"/>
-    <col min="2" max="2" width="17.6328125" customWidth="1"/>
-    <col min="3" max="3" width="15.1796875" customWidth="1"/>
-    <col min="4" max="4" width="11.36328125" customWidth="1"/>
-    <col min="5" max="5" width="15.1796875" customWidth="1"/>
-    <col min="6" max="6" width="14.90625" customWidth="1"/>
+    <col min="1" max="1" width="17.6328125" customWidth="1"/>
+    <col min="2" max="2" width="15.1796875" customWidth="1"/>
+    <col min="3" max="3" width="11.36328125" customWidth="1"/>
+    <col min="4" max="4" width="15.1796875" customWidth="1"/>
+    <col min="5" max="5" width="14.90625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="3" t="s">
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="2" t="s">
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51979F2D-3076-4829-ADC1-FEE540642646}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
         <v>23</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>